<commit_message>
fix(reference-data): restore 188 researched university locations and add 123 cities
</commit_message>
<xml_diff>
--- a/workspace/import-sources/universities/stage-1/Oceania_Universities_Import_English_14_Countries_COMPLETE.xlsx
+++ b/workspace/import-sources/universities/stage-1/Oceania_Universities_Import_English_14_Countries_COMPLETE.xlsx
@@ -731,7 +731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P71"/>
+  <dimension ref="A1:P72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5691,7 +5691,83 @@
         </is>
       </c>
     </row>
-    <row r="72" ht="28" customHeight="1"/>
+    <row r="72" ht="28" customHeight="1">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>INS-AUS-0023</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>University of the Sunshine Coast</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>University of the Sunshine Coast</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>AUS</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Sippy Downs</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>University</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>https://www.usc.edu.au/</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>https://www.teqsa.gov.au/national-register | https://universitiesaustralia.edu.au/our-universities/university-profiles/</t>
+        </is>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>city_au_official_sippy_downs</t>
+        </is>
+      </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>AU-QLD</t>
+        </is>
+      </c>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t>SOURCE_MATCHED</t>
+        </is>
+      </c>
+      <c r="P72" t="inlineStr">
+        <is>
+          <t>PRIMARY_ADDRESS_SEARCH_INDEX_NOT_LIVE_VERIFIED</t>
+        </is>
+      </c>
+    </row>
     <row r="73" ht="28" customHeight="1"/>
   </sheetData>
   <mergeCells count="2">
@@ -6921,7 +6997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P3"/>
+  <dimension ref="A1:P2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7009,37 +7085,37 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>INS-AUS-0023</t>
+          <t>INS-PNG-0004</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>University of the Sunshine Coast</t>
+          <t>Papua New Guinea University of Natural Resources and Environment</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>University of the Sunshine Coast</t>
+          <t>Papua New Guinea University of Natural Resources and Environment</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Papua New Guinea</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>AUS</t>
+          <t>PNG</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Sippy Downs</t>
+          <t>Vudal</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>University</t>
+          <t>Agricultural University</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -7054,12 +7130,12 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>https://www.usc.edu.au/</t>
+          <t>https://www.unre.ac.pg/</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>https://www.teqsa.gov.au/national-register | https://universitiesaustralia.edu.au/our-universities/university-profiles/</t>
+          <t>https://apply.dherst.gov.pg/ | https://web.dherst.gov.pg/</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -7068,73 +7144,6 @@
         </is>
       </c>
       <c r="P2" t="inlineStr">
-        <is>
-          <t>OFFICIAL_ADDRESS_NOT_YET_CORROBORATED</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>INS-PNG-0004</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Papua New Guinea University of Natural Resources and Environment</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Papua New Guinea University of Natural Resources and Environment</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Papua New Guinea</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>PNG</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Vudal</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Agricultural University</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Public</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>https://www.unre.ac.pg/</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>https://apply.dherst.gov.pg/ | https://web.dherst.gov.pg/</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>REVIEW_REQUIRED</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
         <is>
           <t>OFFICIAL_ADDRESS_NOT_YET_CORROBORATED</t>
         </is>

</xml_diff>

<commit_message>
fix(reference-data): apply reviewed university location workbook batch 12
</commit_message>
<xml_diff>
--- a/workspace/import-sources/universities/stage-1/Oceania_Universities_Import_English_14_Countries_COMPLETE.xlsx
+++ b/workspace/import-sources/universities/stage-1/Oceania_Universities_Import_English_14_Countries_COMPLETE.xlsx
@@ -731,7 +731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P72"/>
+  <dimension ref="A1:P73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -784,7 +784,6 @@
       <c r="K2" s="1" t="n"/>
       <c r="L2" s="1" t="n"/>
     </row>
-    <row r="3"/>
     <row r="4" ht="32" customHeight="1">
       <c r="A4" s="26" t="inlineStr">
         <is>
@@ -5768,7 +5767,83 @@
         </is>
       </c>
     </row>
-    <row r="73" ht="28" customHeight="1"/>
+    <row r="73" ht="28" customHeight="1">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>INS-PNG-0004</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Papua New Guinea University of Natural Resources and Environment</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Papua New Guinea University of Natural Resources and Environment</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Papua New Guinea</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>PNG</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Vudal</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Agricultural University</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>https://www.unre.ac.pg/</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>https://apply.dherst.gov.pg/ | https://web.dherst.gov.pg/</t>
+        </is>
+      </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>city_pg_official_vudal</t>
+        </is>
+      </c>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>PG-EBR</t>
+        </is>
+      </c>
+      <c r="O73" t="inlineStr">
+        <is>
+          <t>SOURCE_MATCHED</t>
+        </is>
+      </c>
+      <c r="P73" t="inlineStr">
+        <is>
+          <t>USER_RESEARCH_ADDRESS_REQUIRES_OWNER_VERIFICATION</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:L2"/>
@@ -6997,7 +7072,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:P1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7082,73 +7157,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>INS-PNG-0004</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Papua New Guinea University of Natural Resources and Environment</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Papua New Guinea University of Natural Resources and Environment</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Papua New Guinea</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>PNG</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Vudal</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Agricultural University</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Public</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>https://www.unre.ac.pg/</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>https://apply.dherst.gov.pg/ | https://web.dherst.gov.pg/</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>REVIEW_REQUIRED</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>OFFICIAL_ADDRESS_NOT_YET_CORROBORATED</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>